<commit_message>
Altium generated BOMs added. Input Boards and LED round board revised.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Altium_Generated/Input_Board.xlsx
+++ b/Deliverables/BOM/Altium_Generated/Input_Board.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\IbrahimHyder-ReverseEngineering\Deliverables\BOM\Altium_Generated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{92F6D473-10E6-4D99-A299-0BEFDE073736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{50A9848B-F2B7-4DC5-AF21-6D05F4329D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2685" yWindow="300" windowWidth="10335" windowHeight="10620" xr2:uid="{1AFB325F-3F09-4048-91DB-2C4A4B65E6BA}"/>
+    <workbookView xWindow="10155" yWindow="300" windowWidth="10335" windowHeight="10620" xr2:uid="{02904BEF-D4A7-4E5E-9EDD-031991C7BC06}"/>
   </bookViews>
   <sheets>
     <sheet name="Input_Board" sheetId="1" r:id="rId1"/>
@@ -454,7 +454,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C87E5A81-07AA-48C6-A178-547DBE17BE4D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3F1E0E2-5B94-4DF4-AB3C-3C38AD0FB3EC}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>

</xml_diff>

<commit_message>
Changes in Altium generated and DigiKey BOM of Input Board of Ibrahim.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Altium_Generated/Input_Board.xlsx
+++ b/Deliverables/BOM/Altium_Generated/Input_Board.xlsx
@@ -5,20 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\IbrahimHyder-ReverseEngineering\Deliverables\BOM\Altium_Generated\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eSpark-37\Documents\GitHub\IbrahimHyder-ReverseEngineering\Deliverables\BOM\Altium_Generated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{50A9848B-F2B7-4DC5-AF21-6D05F4329D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB0A55E7-38F4-47CB-ABAE-1903103267D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10155" yWindow="300" windowWidth="10335" windowHeight="10620" xr2:uid="{02904BEF-D4A7-4E5E-9EDD-031991C7BC06}"/>
+    <workbookView xWindow="-15" yWindow="7365" windowWidth="19230" windowHeight="7410" xr2:uid="{5A2D0F1A-2CA0-4032-AB19-95CD7F58DF92}"/>
   </bookViews>
   <sheets>
     <sheet name="Input_Board" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">Input_Board!$1:$1</definedName>
-  </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
   <si>
     <t>Comment</t>
   </si>
@@ -42,13 +39,16 @@
     <t>Footprint</t>
   </si>
   <si>
-    <t>LibRef</t>
+    <t>Manufacturer</t>
   </si>
   <si>
     <t>Quantity</t>
   </si>
   <si>
-    <t>Manufacturer</t>
+    <t>Value</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>S2B-PH-K-S(LF)(SN)</t>
@@ -63,26 +63,95 @@
     <t>JST</t>
   </si>
   <si>
-    <t>DC-005-5A-2.5-SMT</t>
-  </si>
-  <si>
-    <t>DC Power Receptacle Jack 2.5A 2.5mm 6.5mm SMD Power Connectors RoHS</t>
+    <t>U262-241N-4BVC16</t>
+  </si>
+  <si>
+    <t>Receptacle USB - Type C 24 - Sinking board USB Connectors ROHS</t>
   </si>
   <si>
     <t>J2</t>
   </si>
   <si>
-    <t>XKB Enterprise</t>
+    <t>XKB Connectivity</t>
+  </si>
+  <si>
+    <t>Test Point ON</t>
+  </si>
+  <si>
+    <t>P1, P2, P3, P4, P5, P6</t>
+  </si>
+  <si>
+    <t>5.1K</t>
+  </si>
+  <si>
+    <t>RES 5.1K OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>R1, R2</t>
+  </si>
+  <si>
+    <t>Res0603</t>
+  </si>
+  <si>
+    <t>RMCF0603FT5K10</t>
+  </si>
+  <si>
+    <t>Stackpole Electronics</t>
+  </si>
+  <si>
+    <t>S. No.</t>
+  </si>
+  <si>
+    <t>Bill of Material(BOM) for Input Board</t>
+  </si>
+  <si>
+    <t>Manufacturer Part No.</t>
+  </si>
+  <si>
+    <t>---</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Connectors</t>
+  </si>
+  <si>
+    <t>Custom(SMD)</t>
+  </si>
+  <si>
+    <t>Do Not Mount</t>
+  </si>
+  <si>
+    <t>Through Hole (2.0mm)</t>
+  </si>
+  <si>
+    <t>Resistors</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -97,12 +166,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD3D3D3"/>
+        <fgColor indexed="22"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -125,21 +194,278 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -454,89 +780,202 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3F1E0E2-5B94-4DF4-AB3C-3C38AD0FB3EC}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:G3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B31A00A8-0DA4-4D58-A5BE-A5B8774082CA}">
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="6" width="19.7109375" customWidth="1"/>
-    <col min="7" max="7" width="16.5703125" customWidth="1"/>
+    <col min="1" max="1" width="7" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16.140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="8.7109375" style="2" customWidth="1"/>
+    <col min="9" max="9" width="6.5703125" style="4" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="25"/>
+    </row>
+    <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="26"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="28"/>
+    </row>
+    <row r="3" spans="1:10" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I3" s="6" t="s">
         <v>6</v>
       </c>
+      <c r="J3" s="13" t="s">
+        <v>28</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+    <row r="4" spans="1:10" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="14">
+        <v>1</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="9">
+        <v>2</v>
+      </c>
+      <c r="I4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="J4" s="15"/>
+    </row>
+    <row r="5" spans="1:10" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="14">
+        <v>2</v>
+      </c>
+      <c r="B5" s="30"/>
+      <c r="C5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="9">
+        <v>1</v>
+      </c>
+      <c r="I5" s="10"/>
+      <c r="J5" s="15"/>
+    </row>
+    <row r="6" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="14">
+        <v>3</v>
+      </c>
+      <c r="B6" s="31"/>
+      <c r="C6" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="9">
+        <v>6</v>
+      </c>
+      <c r="I6" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="4">
+      <c r="J6" s="15" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" s="3" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="16">
+        <v>4</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="19">
         <v>2</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="4">
-        <v>1</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>14</v>
-      </c>
+      <c r="I7" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" s="21"/>
     </row>
   </sheetData>
-  <printOptions horizontalCentered="1" verticalCentered="1"/>
-  <pageMargins left="0.30555555555555558" right="0.30555555555555558" top="0.30555555555555558" bottom="0.30555555555555558" header="0" footer="0"/>
-  <pageSetup scale="98" orientation="landscape" blackAndWhite="1" r:id="rId1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J2"/>
+    <mergeCell ref="B4:B6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>